<commit_message>
#16 Transformer Price remove from eSpark BOM
</commit_message>
<xml_diff>
--- a/Design-Files/OFP_VIM_v1.5/BOM/eSpark-BOM-OFP_VIM_v1.5.xlsx
+++ b/Design-Files/OFP_VIM_v1.5/BOM/eSpark-BOM-OFP_VIM_v1.5.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="10 Boards" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1087" uniqueCount="382">
   <si>
     <t>Component list</t>
   </si>
@@ -4561,12 +4561,11 @@
       <c r="O51" s="44" t="s">
         <v>280</v>
       </c>
-      <c r="P51" s="21">
-        <v>3</v>
-      </c>
-      <c r="Q51" s="21">
-        <f t="shared" si="22"/>
-        <v>33</v>
+      <c r="P51" s="21" t="s">
+        <v>280</v>
+      </c>
+      <c r="Q51" s="21" t="s">
+        <v>280</v>
       </c>
       <c r="R51" s="14"/>
     </row>
@@ -4756,7 +4755,7 @@
       <c r="P55" s="50"/>
       <c r="Q55" s="18">
         <f>SUM(Q8:Q54)</f>
-        <v>196.70939999999999</v>
+        <v>163.70939999999999</v>
       </c>
       <c r="R55" s="1"/>
     </row>
@@ -4781,7 +4780,7 @@
       <c r="P56" s="50"/>
       <c r="Q56" s="19">
         <f>Q55/10</f>
-        <v>19.670939999999998</v>
+        <v>16.370939999999997</v>
       </c>
       <c r="R56" s="1"/>
     </row>
@@ -7461,12 +7460,11 @@
       <c r="O51" s="44" t="s">
         <v>280</v>
       </c>
-      <c r="P51" s="21">
-        <v>0.93</v>
-      </c>
-      <c r="Q51" s="21">
-        <f t="shared" si="22"/>
-        <v>931.86</v>
+      <c r="P51" s="21" t="s">
+        <v>280</v>
+      </c>
+      <c r="Q51" s="21" t="s">
+        <v>280</v>
       </c>
       <c r="R51" s="14"/>
     </row>
@@ -7656,7 +7654,7 @@
       <c r="P55" s="50"/>
       <c r="Q55" s="18">
         <f>SUM(Q8:Q54)</f>
-        <v>9710.8852999999999</v>
+        <v>8779.0253000000012</v>
       </c>
       <c r="R55" s="1"/>
     </row>
@@ -7681,7 +7679,7 @@
       <c r="P56" s="50"/>
       <c r="Q56" s="19">
         <f>Q55/1000</f>
-        <v>9.7108852999999993</v>
+        <v>8.7790253000000007</v>
       </c>
       <c r="R56" s="1"/>
     </row>

</xml_diff>